<commit_message>
Update benchmark_results.xlsx with complete HumanEval data for all models
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/benchmark_results.xlsx
+++ b/benchmark_results.xlsx
@@ -135,10 +135,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N88"/>
+  <dimension ref="A1:J88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1886,10 +1886,8 @@
       <c r="I41" s="4" t="n">
         <v>1.67</v>
       </c>
-      <c r="J41" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J41" s="4" t="n">
+        <v>0.616</v>
       </c>
     </row>
     <row r="42">
@@ -1918,10 +1916,8 @@
       <c r="I42" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="J42" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J42" s="6" t="n">
+        <v>0.604</v>
       </c>
     </row>
     <row r="43">
@@ -1950,10 +1946,8 @@
       <c r="I43" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="J43" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J43" s="8" t="n">
+        <v>0.628</v>
       </c>
     </row>
     <row r="44">
@@ -1990,10 +1984,8 @@
       <c r="I44" s="4" t="n">
         <v>1.5</v>
       </c>
-      <c r="J44" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J44" s="4" t="n">
+        <v>0.616</v>
       </c>
     </row>
     <row r="45">
@@ -2022,10 +2014,8 @@
       <c r="I45" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="J45" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J45" s="6" t="n">
+        <v>0.604</v>
       </c>
     </row>
     <row r="46">
@@ -2054,10 +2044,8 @@
       <c r="I46" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="J46" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J46" s="8" t="n">
+        <v>0.628</v>
       </c>
     </row>
     <row r="47">
@@ -2094,10 +2082,8 @@
       <c r="I47" s="4" t="n">
         <v>3.67</v>
       </c>
-      <c r="J47" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J47" s="4" t="n">
+        <v>0.616</v>
       </c>
     </row>
     <row r="48">
@@ -2126,10 +2112,8 @@
       <c r="I48" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="J48" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J48" s="6" t="n">
+        <v>0.604</v>
       </c>
     </row>
     <row r="49">
@@ -2158,10 +2142,8 @@
       <c r="I49" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="J49" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J49" s="8" t="n">
+        <v>0.628</v>
       </c>
     </row>
     <row r="50">
@@ -2198,10 +2180,8 @@
       <c r="I50" s="4" t="n">
         <v>2.07</v>
       </c>
-      <c r="J50" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J50" s="4" t="n">
+        <v>0.8110000000000001</v>
       </c>
     </row>
     <row r="51">
@@ -2230,10 +2210,8 @@
       <c r="I51" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="J51" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J51" s="6" t="n">
+        <v>0.768</v>
       </c>
     </row>
     <row r="52">
@@ -2262,10 +2240,8 @@
       <c r="I52" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="J52" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J52" s="8" t="n">
+        <v>0.805</v>
       </c>
     </row>
     <row r="53">
@@ -2302,10 +2278,8 @@
       <c r="I53" s="4" t="n">
         <v>1.53</v>
       </c>
-      <c r="J53" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J53" s="4" t="n">
+        <v>0.8110000000000001</v>
       </c>
     </row>
     <row r="54">
@@ -2334,10 +2308,8 @@
       <c r="I54" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="J54" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J54" s="6" t="n">
+        <v>0.768</v>
       </c>
     </row>
     <row r="55">
@@ -2366,10 +2338,8 @@
       <c r="I55" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="J55" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J55" s="8" t="n">
+        <v>0.805</v>
       </c>
     </row>
     <row r="56">
@@ -2406,10 +2376,8 @@
       <c r="I56" s="4" t="n">
         <v>1.8</v>
       </c>
-      <c r="J56" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J56" s="4" t="n">
+        <v>0.835</v>
       </c>
     </row>
     <row r="57">
@@ -2438,10 +2406,8 @@
       <c r="I57" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="J57" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J57" s="6" t="n">
+        <v>0.829</v>
       </c>
     </row>
     <row r="58">
@@ -2470,10 +2436,8 @@
       <c r="I58" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="J58" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J58" s="8" t="n">
+        <v>0.835</v>
       </c>
     </row>
     <row r="59">
@@ -2510,10 +2474,8 @@
       <c r="I59" s="4" t="n">
         <v>1.6</v>
       </c>
-      <c r="J59" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J59" s="4" t="n">
+        <v>0.835</v>
       </c>
     </row>
     <row r="60">
@@ -2542,10 +2504,8 @@
       <c r="I60" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="J60" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J60" s="6" t="n">
+        <v>0.829</v>
       </c>
     </row>
     <row r="61">
@@ -2574,10 +2534,8 @@
       <c r="I61" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="J61" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J61" s="8" t="n">
+        <v>0.835</v>
       </c>
     </row>
     <row r="62">
@@ -2614,10 +2572,8 @@
       <c r="I62" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J62" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J62" s="4" t="n">
+        <v>0.835</v>
       </c>
     </row>
     <row r="63">
@@ -2646,10 +2602,8 @@
       <c r="I63" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="J63" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J63" s="6" t="n">
+        <v>0.829</v>
       </c>
     </row>
     <row r="64">
@@ -2678,10 +2632,8 @@
       <c r="I64" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="J64" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J64" s="8" t="n">
+        <v>0.835</v>
       </c>
     </row>
     <row r="65">
@@ -2718,10 +2670,8 @@
       <c r="I65" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J65" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J65" s="4" t="n">
+        <v>0.908</v>
       </c>
     </row>
     <row r="66">
@@ -2750,10 +2700,8 @@
       <c r="I66" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="J66" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J66" s="6" t="n">
+        <v>0.9330000000000001</v>
       </c>
     </row>
     <row r="67">
@@ -2782,10 +2730,8 @@
       <c r="I67" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="J67" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J67" s="8" t="n">
+        <v>0.896</v>
       </c>
     </row>
     <row r="68">
@@ -2822,10 +2768,8 @@
       <c r="I68" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J68" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J68" s="4" t="n">
+        <v>0.908</v>
       </c>
     </row>
     <row r="69">
@@ -2854,10 +2798,8 @@
       <c r="I69" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="J69" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J69" s="6" t="n">
+        <v>0.9330000000000001</v>
       </c>
     </row>
     <row r="70">
@@ -2886,10 +2828,8 @@
       <c r="I70" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="J70" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J70" s="8" t="n">
+        <v>0.896</v>
       </c>
     </row>
     <row r="71">
@@ -2926,10 +2866,8 @@
       <c r="I71" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J71" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J71" s="4" t="n">
+        <v>0.908</v>
       </c>
     </row>
     <row r="72">
@@ -2958,10 +2896,8 @@
       <c r="I72" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="J72" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J72" s="6" t="n">
+        <v>0.9330000000000001</v>
       </c>
     </row>
     <row r="73">
@@ -2990,10 +2926,8 @@
       <c r="I73" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="J73" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J73" s="8" t="n">
+        <v>0.896</v>
       </c>
     </row>
     <row r="74">
@@ -3030,10 +2964,8 @@
       <c r="I74" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J74" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J74" s="4" t="n">
+        <v>0.908</v>
       </c>
     </row>
     <row r="75">
@@ -3062,10 +2994,8 @@
       <c r="I75" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="J75" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J75" s="6" t="n">
+        <v>0.9330000000000001</v>
       </c>
     </row>
     <row r="76">
@@ -3094,10 +3024,8 @@
       <c r="I76" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="J76" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="J76" s="8" t="n">
+        <v>0.896</v>
       </c>
     </row>
     <row r="77">
@@ -3500,7 +3428,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="A1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3512,7 +3440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3520,6 +3448,7 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3555,6 +3484,11 @@
           <t>Best Pipeline</t>
         </is>
       </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Margin</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -3565,15 +3499,20 @@
       <c r="B3" s="11" t="n">
         <v>0.842</v>
       </c>
-      <c r="C3" s="11" t="n">
+      <c r="C3" s="12" t="n">
         <v>0.8110000000000001</v>
       </c>
-      <c r="D3" s="11" t="n">
+      <c r="D3" s="12" t="n">
         <v>0.835</v>
       </c>
-      <c r="E3" s="12" t="inlineStr">
+      <c r="E3" s="11" t="inlineStr">
         <is>
           <t>iterative</t>
+        </is>
+      </c>
+      <c r="F3" s="12" t="inlineStr">
+        <is>
+          <t>+0.7%</t>
         </is>
       </c>
     </row>
@@ -3583,7 +3522,7 @@
           <t>gemma3:27b</t>
         </is>
       </c>
-      <c r="B4" s="14" t="n">
+      <c r="B4" s="11" t="n">
         <v>0.878</v>
       </c>
       <c r="C4" s="14" t="n">
@@ -3592,9 +3531,14 @@
       <c r="D4" s="14" t="n">
         <v>0.86</v>
       </c>
-      <c r="E4" s="12" t="inlineStr">
+      <c r="E4" s="11" t="inlineStr">
         <is>
           <t>iterative</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>+1.8%</t>
         </is>
       </c>
     </row>
@@ -3604,45 +3548,159 @@
           <t>gpt-oss:20b</t>
         </is>
       </c>
-      <c r="B5" s="11" t="n">
+      <c r="B5" s="12" t="n">
         <v>0.945</v>
       </c>
       <c r="C5" s="11" t="n">
         <v>0.951</v>
       </c>
-      <c r="D5" s="11" t="n">
+      <c r="D5" s="12" t="n">
         <v>0.9330000000000001</v>
       </c>
-      <c r="E5" s="12" t="inlineStr">
+      <c r="E5" s="11" t="inlineStr">
         <is>
           <t>batch</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>+0.6%</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="13" t="inlineStr">
         <is>
+          <t>llama3.1:8b</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="n">
+        <v>0.616</v>
+      </c>
+      <c r="C6" s="14" t="n">
+        <v>0.604</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>0.628</v>
+      </c>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>notdd</t>
+        </is>
+      </c>
+      <c r="F6" s="14" t="inlineStr">
+        <is>
+          <t>+1.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>qwen2.5-coder:3b</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="n">
+        <v>0.8110000000000001</v>
+      </c>
+      <c r="C7" s="12" t="n">
+        <v>0.768</v>
+      </c>
+      <c r="D7" s="12" t="n">
+        <v>0.805</v>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>iterative</t>
+        </is>
+      </c>
+      <c r="F7" s="12" t="inlineStr">
+        <is>
+          <t>+0.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>qwen2.5-coder:7b</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="n">
+        <v>0.835</v>
+      </c>
+      <c r="C8" s="14" t="n">
+        <v>0.829</v>
+      </c>
+      <c r="D8" s="14" t="n">
+        <v>0.835</v>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>iterative</t>
+        </is>
+      </c>
+      <c r="F8" s="14" t="inlineStr">
+        <is>
+          <t>+0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>qwen3:4b</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="n">
+        <v>0.908</v>
+      </c>
+      <c r="C9" s="11" t="n">
+        <v>0.9330000000000001</v>
+      </c>
+      <c r="D9" s="12" t="n">
+        <v>0.896</v>
+      </c>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>batch</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>+2.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
           <t>qwen3:8b</t>
         </is>
       </c>
-      <c r="B6" s="14" t="n">
+      <c r="B10" s="11" t="n">
         <v>0.884</v>
       </c>
-      <c r="C6" s="14" t="n">
+      <c r="C10" s="14" t="n">
         <v>0.872</v>
       </c>
-      <c r="D6" s="14" t="n">
+      <c r="D10" s="14" t="n">
         <v>0.842</v>
       </c>
-      <c r="E6" s="12" t="inlineStr">
+      <c r="E10" s="11" t="inlineStr">
         <is>
           <t>iterative</t>
+        </is>
+      </c>
+      <c r="F10" s="14" t="inlineStr">
+        <is>
+          <t>+1.2%</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3659,15 +3717,15 @@
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
-          <t>Iterative vs Batch vs NoTDD — pass@1 per Model &amp; Preset</t>
+          <t>Iterative vs Batch vs NoTDD — pass@1</t>
         </is>
       </c>
     </row>
@@ -3684,17 +3742,17 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Iterative pass@1</t>
+          <t>Iterative</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Batch pass@1</t>
+          <t>Batch</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>NoTDD pass@1</t>
+          <t>NoTDD</t>
         </is>
       </c>
     </row>
@@ -3709,13 +3767,13 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="C3" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" s="11" t="n">
+      <c r="C3" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="12" t="n">
         <v>0.8</v>
       </c>
-      <c r="E3" s="11" t="n">
+      <c r="E3" s="12" t="n">
         <v>0.9333</v>
       </c>
     </row>
@@ -3730,13 +3788,13 @@
           <t>hard</t>
         </is>
       </c>
-      <c r="C4" s="12" t="n">
+      <c r="C4" s="11" t="n">
         <v>1</v>
       </c>
       <c r="D4" s="14" t="n">
         <v>0.8667</v>
       </c>
-      <c r="E4" s="12" t="n">
+      <c r="E4" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3751,13 +3809,13 @@
           <t>very_hard</t>
         </is>
       </c>
-      <c r="C5" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" s="12" t="n">
+      <c r="C5" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3772,7 +3830,7 @@
           <t>extremely_hard</t>
         </is>
       </c>
-      <c r="C6" s="12" t="n">
+      <c r="C6" s="11" t="n">
         <v>1</v>
       </c>
       <c r="D6" s="14" t="n">
@@ -3793,13 +3851,13 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="C7" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" s="12" t="n">
+      <c r="C7" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3814,13 +3872,13 @@
           <t>hard</t>
         </is>
       </c>
-      <c r="C8" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" s="12" t="n">
+      <c r="C8" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3835,13 +3893,13 @@
           <t>very_hard</t>
         </is>
       </c>
-      <c r="C9" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" s="11" t="n">
+      <c r="C9" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="12" t="n">
         <v>0.9</v>
       </c>
-      <c r="E9" s="12" t="n">
+      <c r="E9" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3856,13 +3914,13 @@
           <t>hard</t>
         </is>
       </c>
-      <c r="C10" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D10" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E10" s="12" t="n">
+      <c r="C10" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3877,13 +3935,13 @@
           <t>very_hard</t>
         </is>
       </c>
-      <c r="C11" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D11" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" s="12" t="n">
+      <c r="C11" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3898,13 +3956,13 @@
           <t>extremely_hard</t>
         </is>
       </c>
-      <c r="C12" s="12" t="n">
+      <c r="C12" s="11" t="n">
         <v>1</v>
       </c>
       <c r="D12" s="14" t="n">
         <v>0.9</v>
       </c>
-      <c r="E12" s="12" t="n">
+      <c r="E12" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3919,13 +3977,13 @@
           <t>hard</t>
         </is>
       </c>
-      <c r="C13" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D13" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" s="11" t="n">
+      <c r="C13" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="12" t="n">
         <v>0.95</v>
       </c>
     </row>
@@ -3940,13 +3998,13 @@
           <t>very_hard</t>
         </is>
       </c>
-      <c r="C14" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D14" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="12" t="n">
+      <c r="C14" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3961,13 +4019,13 @@
           <t>extremely_hard</t>
         </is>
       </c>
-      <c r="C15" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" s="11" t="n">
+      <c r="C15" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="12" t="n">
         <v>0.9</v>
       </c>
-      <c r="E15" s="11" t="n">
+      <c r="E15" s="12" t="n">
         <v>0.9</v>
       </c>
     </row>
@@ -3985,7 +4043,7 @@
       <c r="C16" s="14" t="n">
         <v>0.8667</v>
       </c>
-      <c r="D16" s="12" t="n">
+      <c r="D16" s="11" t="n">
         <v>0.9333</v>
       </c>
       <c r="E16" s="14" t="n">
@@ -4003,13 +4061,13 @@
           <t>hard</t>
         </is>
       </c>
-      <c r="C17" s="11" t="n">
+      <c r="C17" s="12" t="n">
         <v>0.9</v>
       </c>
-      <c r="D17" s="12" t="n">
+      <c r="D17" s="11" t="n">
         <v>0.95</v>
       </c>
-      <c r="E17" s="11" t="n">
+      <c r="E17" s="12" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -4024,13 +4082,13 @@
           <t>very_hard</t>
         </is>
       </c>
-      <c r="C18" s="12" t="n">
+      <c r="C18" s="11" t="n">
         <v>0.3333</v>
       </c>
-      <c r="D18" s="12" t="n">
+      <c r="D18" s="11" t="n">
         <v>0.3333</v>
       </c>
-      <c r="E18" s="12" t="n">
+      <c r="E18" s="11" t="n">
         <v>0.3333</v>
       </c>
     </row>
@@ -4045,13 +4103,13 @@
           <t>easy</t>
         </is>
       </c>
-      <c r="C19" s="11" t="n">
+      <c r="C19" s="12" t="n">
         <v>0.7333</v>
       </c>
-      <c r="D19" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E19" s="11" t="n">
+      <c r="D19" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="12" t="n">
         <v>0.7333</v>
       </c>
     </row>
@@ -4066,13 +4124,13 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="C20" s="12" t="n">
+      <c r="C20" s="11" t="n">
         <v>0.8667</v>
       </c>
       <c r="D20" s="14" t="n">
         <v>0.7333</v>
       </c>
-      <c r="E20" s="12" t="n">
+      <c r="E20" s="11" t="n">
         <v>0.8667</v>
       </c>
     </row>
@@ -4087,13 +4145,13 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="C21" s="11" t="n">
+      <c r="C21" s="12" t="n">
         <v>0.8</v>
       </c>
-      <c r="D21" s="12" t="n">
+      <c r="D21" s="11" t="n">
         <v>0.9333</v>
       </c>
-      <c r="E21" s="11" t="n">
+      <c r="E21" s="12" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -4111,7 +4169,7 @@
       <c r="C22" s="14" t="n">
         <v>0.85</v>
       </c>
-      <c r="D22" s="12" t="n">
+      <c r="D22" s="11" t="n">
         <v>0.95</v>
       </c>
       <c r="E22" s="14" t="n">
@@ -4129,13 +4187,13 @@
           <t>very_hard</t>
         </is>
       </c>
-      <c r="C23" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D23" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E23" s="12" t="n">
+      <c r="C23" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4150,13 +4208,13 @@
           <t>easy</t>
         </is>
       </c>
-      <c r="C24" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D24" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E24" s="12" t="n">
+      <c r="C24" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4171,13 +4229,13 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="C25" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D25" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E25" s="12" t="n">
+      <c r="C25" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4192,13 +4250,13 @@
           <t>hard</t>
         </is>
       </c>
-      <c r="C26" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D26" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E26" s="12" t="n">
+      <c r="C26" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4213,13 +4271,13 @@
           <t>very_hard</t>
         </is>
       </c>
-      <c r="C27" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D27" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E27" s="12" t="n">
+      <c r="C27" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4234,13 +4292,13 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="C28" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D28" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E28" s="12" t="n">
+      <c r="C28" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4255,13 +4313,13 @@
           <t>hard</t>
         </is>
       </c>
-      <c r="C29" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D29" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E29" s="12" t="n">
+      <c r="C29" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4276,13 +4334,13 @@
           <t>very_hard</t>
         </is>
       </c>
-      <c r="C30" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D30" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E30" s="12" t="n">
+      <c r="C30" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4297,13 +4355,13 @@
           <t>extremely_hard</t>
         </is>
       </c>
-      <c r="C31" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D31" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E31" s="12" t="n">
+      <c r="C31" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4334,7 +4392,7 @@
     <row r="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
-          <t>Mutation Score — Iterative vs Batch vs NoTDD</t>
+          <t>Mutation Score — Code Quality Comparison</t>
         </is>
       </c>
     </row>
@@ -4376,13 +4434,13 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="C3" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" s="12" t="n">
+      <c r="C3" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4397,13 +4455,13 @@
           <t>hard</t>
         </is>
       </c>
-      <c r="C4" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" s="12" t="n">
+      <c r="C4" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4418,13 +4476,13 @@
           <t>very_hard</t>
         </is>
       </c>
-      <c r="C5" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" s="12" t="n">
+      <c r="C5" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4439,13 +4497,13 @@
           <t>extremely_hard</t>
         </is>
       </c>
-      <c r="C6" s="12" t="n">
+      <c r="C6" s="11" t="n">
         <v>1</v>
       </c>
       <c r="D6" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="12" t="n">
+      <c r="E6" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4460,13 +4518,13 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="C7" s="11" t="n">
+      <c r="C7" s="12" t="n">
         <v>0.921</v>
       </c>
-      <c r="D7" s="12" t="n">
+      <c r="D7" s="11" t="n">
         <v>0.945</v>
       </c>
-      <c r="E7" s="11" t="n">
+      <c r="E7" s="12" t="n">
         <v>0.9330000000000001</v>
       </c>
     </row>
@@ -4481,10 +4539,10 @@
           <t>hard</t>
         </is>
       </c>
-      <c r="C8" s="12" t="n">
+      <c r="C8" s="11" t="n">
         <v>0.958</v>
       </c>
-      <c r="D8" s="12" t="n">
+      <c r="D8" s="11" t="n">
         <v>0.958</v>
       </c>
       <c r="E8" s="14" t="n">
@@ -4502,13 +4560,13 @@
           <t>very_hard</t>
         </is>
       </c>
-      <c r="C9" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" s="11" t="n">
+      <c r="C9" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="12" t="n">
         <v>0.983</v>
       </c>
-      <c r="E9" s="12" t="n">
+      <c r="E9" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4523,10 +4581,10 @@
           <t>hard</t>
         </is>
       </c>
-      <c r="C10" s="12" t="n">
+      <c r="C10" s="11" t="n">
         <v>0.958</v>
       </c>
-      <c r="D10" s="12" t="n">
+      <c r="D10" s="11" t="n">
         <v>0.958</v>
       </c>
       <c r="E10" s="14" t="n">
@@ -4544,13 +4602,13 @@
           <t>very_hard</t>
         </is>
       </c>
-      <c r="C11" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D11" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" s="12" t="n">
+      <c r="C11" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4568,7 +4626,7 @@
       <c r="C12" s="14" t="n">
         <v>0.757</v>
       </c>
-      <c r="D12" s="12" t="n">
+      <c r="D12" s="11" t="n">
         <v>0.836</v>
       </c>
       <c r="E12" s="14" t="n">
@@ -4586,13 +4644,13 @@
           <t>hard</t>
         </is>
       </c>
-      <c r="C13" s="11" t="n">
+      <c r="C13" s="12" t="n">
         <v>0.873</v>
       </c>
-      <c r="D13" s="12" t="n">
+      <c r="D13" s="11" t="n">
         <v>0.949</v>
       </c>
-      <c r="E13" s="11" t="n">
+      <c r="E13" s="12" t="n">
         <v>0.897</v>
       </c>
     </row>
@@ -4613,7 +4671,7 @@
       <c r="D14" s="14" t="n">
         <v>0.75</v>
       </c>
-      <c r="E14" s="12" t="n">
+      <c r="E14" s="11" t="n">
         <v>0.955</v>
       </c>
     </row>
@@ -4628,13 +4686,13 @@
           <t>extremely_hard</t>
         </is>
       </c>
-      <c r="C15" s="11" t="n">
+      <c r="C15" s="12" t="n">
         <v>0.793</v>
       </c>
-      <c r="D15" s="12" t="n">
+      <c r="D15" s="11" t="n">
         <v>0.962</v>
       </c>
-      <c r="E15" s="11" t="n">
+      <c r="E15" s="12" t="n">
         <v>0.82</v>
       </c>
     </row>
@@ -4649,13 +4707,13 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="C16" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E16" s="12" t="n">
+      <c r="C16" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4670,13 +4728,13 @@
           <t>hard</t>
         </is>
       </c>
-      <c r="C17" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E17" s="12" t="n">
+      <c r="C17" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4691,13 +4749,13 @@
           <t>very_hard</t>
         </is>
       </c>
-      <c r="C18" s="12" t="n">
+      <c r="C18" s="11" t="n">
         <v>0.3333</v>
       </c>
-      <c r="D18" s="12" t="n">
+      <c r="D18" s="11" t="n">
         <v>0.3333</v>
       </c>
-      <c r="E18" s="12" t="n">
+      <c r="E18" s="11" t="n">
         <v>0.3333</v>
       </c>
     </row>
@@ -4712,13 +4770,13 @@
           <t>easy</t>
         </is>
       </c>
-      <c r="C19" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E19" s="12" t="n">
+      <c r="C19" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4733,13 +4791,13 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="C20" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E20" s="12" t="n">
+      <c r="C20" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4754,13 +4812,13 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="C21" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D21" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E21" s="12" t="n">
+      <c r="C21" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4775,13 +4833,13 @@
           <t>hard</t>
         </is>
       </c>
-      <c r="C22" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D22" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E22" s="12" t="n">
+      <c r="C22" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4796,13 +4854,13 @@
           <t>very_hard</t>
         </is>
       </c>
-      <c r="C23" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D23" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E23" s="12" t="n">
+      <c r="C23" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4817,13 +4875,13 @@
           <t>easy</t>
         </is>
       </c>
-      <c r="C24" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D24" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E24" s="12" t="n">
+      <c r="C24" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4838,13 +4896,13 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="C25" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D25" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E25" s="12" t="n">
+      <c r="C25" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4859,13 +4917,13 @@
           <t>hard</t>
         </is>
       </c>
-      <c r="C26" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D26" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E26" s="12" t="n">
+      <c r="C26" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4880,13 +4938,13 @@
           <t>very_hard</t>
         </is>
       </c>
-      <c r="C27" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D27" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E27" s="12" t="n">
+      <c r="C27" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4901,13 +4959,13 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="C28" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D28" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E28" s="12" t="n">
+      <c r="C28" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4922,13 +4980,13 @@
           <t>hard</t>
         </is>
       </c>
-      <c r="C29" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D29" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E29" s="12" t="n">
+      <c r="C29" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4943,13 +5001,13 @@
           <t>very_hard</t>
         </is>
       </c>
-      <c r="C30" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D30" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E30" s="12" t="n">
+      <c r="C30" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4964,13 +5022,13 @@
           <t>extremely_hard</t>
         </is>
       </c>
-      <c r="C31" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D31" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E31" s="12" t="n">
+      <c r="C31" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="11" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>